<commit_message>
update, dev can be used again
</commit_message>
<xml_diff>
--- a/notebooks/outputs/building_sector_energy_summary.xlsx
+++ b/notebooks/outputs/building_sector_energy_summary.xlsx
@@ -452,10 +452,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17037388447.40662</v>
+        <v>17037388789.9289</v>
       </c>
       <c r="C2" t="n">
-        <v>4.937597294189578</v>
+        <v>6.825759420813151</v>
       </c>
     </row>
     <row r="3">
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19720127169.47928</v>
+        <v>19720127182.08091</v>
       </c>
       <c r="C3" t="n">
-        <v>5.715080503897102</v>
+        <v>7.900555980285521</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +478,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9715263660.927742</v>
+        <v>10051147245.10204</v>
       </c>
       <c r="C4" t="n">
-        <v>2.81557585615987</v>
+        <v>4.026832623482187</v>
       </c>
     </row>
     <row r="5">
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10854992399.07086</v>
+        <v>10854992275.54213</v>
       </c>
       <c r="C5" t="n">
-        <v>3.145880089753966</v>
+        <v>4.348880377222693</v>
       </c>
     </row>
     <row r="6">
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>48430444582.01988</v>
+        <v>24834532561.80243</v>
       </c>
       <c r="C6" t="n">
-        <v>14.0356036878985</v>
+        <v>9.949561325701326</v>
       </c>
     </row>
     <row r="7">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10738893612.2741</v>
+        <v>10738894002.57796</v>
       </c>
       <c r="C7" t="n">
-        <v>3.112233556582761</v>
+        <v>4.302367446738077</v>
       </c>
     </row>
     <row r="8">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>51983752299.93461</v>
+        <v>51983753921.33759</v>
       </c>
       <c r="C8" t="n">
-        <v>15.06538607664655</v>
+        <v>20.82646598213149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>